<commit_message>
Latest code hungary UI Change Code
</commit_message>
<xml_diff>
--- a/Data/TestDataPoland-Endto End_Passed - Andre update.xlsx
+++ b/Data/TestDataPoland-Endto End_Passed - Andre update.xlsx
@@ -1,32 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{251B5B6A-389C-4668-BCBD-6AD462CC6792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">Sheet1!$A$1:$BY$8</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -191,11 +177,11 @@
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -270,7 +256,7 @@
     <t>Test_17</t>
   </si>
   <si>
-    <t>10697803</t>
+    <t>10697807</t>
   </si>
   <si>
     <t>Passed</t>
@@ -282,10 +268,10 @@
     <t>Poland</t>
   </si>
   <si>
-    <t>Mireille</t>
-  </si>
-  <si>
-    <t>Howe</t>
+    <t>Joshuah</t>
+  </si>
+  <si>
+    <t>Prohaska</t>
   </si>
   <si>
     <t xml:space="preserve">698 980 460 </t>
@@ -381,7 +367,7 @@
     <t>ID Card</t>
   </si>
   <si>
-    <t>GHE456139</t>
+    <t>GSK567484</t>
   </si>
   <si>
     <t>Male</t>
@@ -432,10 +418,10 @@
     <t>Failed</t>
   </si>
   <si>
-    <t>Nayeli</t>
-  </si>
-  <si>
-    <t>Thiel</t>
+    <t>Benny</t>
+  </si>
+  <si>
+    <t>Trantow</t>
   </si>
   <si>
     <t>In-Store Visual Merchandising Assistant_NEW</t>
@@ -552,127 +538,127 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color rgb="FFFF0000"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <color indexed="8"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color indexed="8"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color indexed="8"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color indexed="8"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
+      <color indexed="63"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color indexed="63"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
+      <color indexed="12"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color indexed="12"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <color indexed="8"/>
+      <family val="2"/>
       <sz val="14"/>
-      <color indexed="8"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <color indexed="10"/>
+      <family val="2"/>
       <sz val="14"/>
-      <color indexed="10"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFFF0000"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
       <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
-      <sz val="16"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="16"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <family val="2"/>
+      <scheme val="minor"/>
       <sz val="16"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
+      <color rgb="FF000000"/>
+      <family val="2"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -684,7 +670,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -715,18 +701,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
     <border>
@@ -736,12 +714,8 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1153,9 +1127,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:BY8"/>
-  <sheetFormatPr defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="10.81640625" customWidth="1"/>
     <col min="2" max="2" width="156.54296875" customWidth="1"/>
@@ -1224,7 +1198,7 @@
     <col min="77" max="77" width="26.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:77" s="2" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" ht="35" customHeight="1" spans="1:77" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1457,7 +1431,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:77" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="52.5" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -1489,7 +1463,7 @@
         <v>83</v>
       </c>
       <c r="K2" s="33">
-        <f t="shared" ref="K2:K3" ca="1" si="0">TODAY()-31</f>
+        <f t="shared" ref="K2:K3" si="0">TODAY()-31</f>
         <v>45692</v>
       </c>
       <c r="L2" s="34" t="s">
@@ -1529,7 +1503,7 @@
         <v>83</v>
       </c>
       <c r="X2" s="33">
-        <f t="shared" ref="X2:X8" ca="1" si="1">K2</f>
+        <f t="shared" ref="X2:X8" si="1">K2</f>
         <v>45692</v>
       </c>
       <c r="Y2" s="34" t="s">
@@ -1575,7 +1549,7 @@
         <v>98</v>
       </c>
       <c r="AM2" s="36">
-        <f t="shared" ref="AM2" ca="1" si="2">TODAY()+365</f>
+        <f t="shared" ref="AM2" si="2">TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AN2" s="34">
@@ -1591,15 +1565,15 @@
         <v>101</v>
       </c>
       <c r="AR2" s="33">
-        <f t="shared" ref="AR2:AR8" ca="1" si="3">X2</f>
+        <f t="shared" ref="AR2:AR8" si="3">X2</f>
         <v>45692</v>
       </c>
       <c r="AS2" s="33">
-        <f t="shared" ref="AS2:AS8" ca="1" si="4">X2</f>
+        <f t="shared" ref="AS2:AS8" si="4">X2</f>
         <v>45692</v>
       </c>
       <c r="AT2" s="36">
-        <f t="shared" ref="AT2" ca="1" si="5">TODAY()+365</f>
+        <f t="shared" ref="AT2" si="5">TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AU2" s="34" t="s">
@@ -1634,7 +1608,7 @@
         <v>109</v>
       </c>
       <c r="BF2" s="15">
-        <v>9477896627</v>
+        <v>7477896627</v>
       </c>
       <c r="BG2" s="31" t="s">
         <v>78</v>
@@ -1643,7 +1617,7 @@
         <v>110</v>
       </c>
       <c r="BI2" s="15">
-        <v>47678965361</v>
+        <v>57678965361</v>
       </c>
       <c r="BJ2" s="31" t="s">
         <v>78</v>
@@ -1694,7 +1668,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:77" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="52.5" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -1726,7 +1700,7 @@
         <v>83</v>
       </c>
       <c r="K3" s="33">
-        <f t="shared" ca="1" si="0"/>
+        <f t="shared" si="0"/>
         <v>45692</v>
       </c>
       <c r="L3" s="34" t="s">
@@ -1766,7 +1740,7 @@
         <v>83</v>
       </c>
       <c r="X3" s="33">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45692</v>
       </c>
       <c r="Y3" s="34" t="s">
@@ -1812,7 +1786,7 @@
         <v>98</v>
       </c>
       <c r="AM3" s="33">
-        <f t="shared" ref="AM3:AM5" ca="1" si="6">TODAY()+365</f>
+        <f t="shared" ref="AM3:AM5" si="6">TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AN3" s="34">
@@ -1828,11 +1802,11 @@
         <v>101</v>
       </c>
       <c r="AR3" s="33">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45692</v>
       </c>
       <c r="AS3" s="33">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45692</v>
       </c>
       <c r="AT3" s="33" t="s">
@@ -1930,7 +1904,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="4" spans="1:77" ht="54" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="4" ht="54" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -1962,7 +1936,7 @@
         <v>83</v>
       </c>
       <c r="K4" s="33">
-        <f ca="1">TODAY()+91</f>
+        <f>TODAY()+91</f>
         <v>45814</v>
       </c>
       <c r="L4" s="34" t="s">
@@ -2002,7 +1976,7 @@
         <v>83</v>
       </c>
       <c r="X4" s="33">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45814</v>
       </c>
       <c r="Y4" s="34" t="s">
@@ -2048,7 +2022,7 @@
         <v>98</v>
       </c>
       <c r="AM4" s="33">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>46088</v>
       </c>
       <c r="AN4" s="34">
@@ -2064,11 +2038,11 @@
         <v>101</v>
       </c>
       <c r="AR4" s="33">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45814</v>
       </c>
       <c r="AS4" s="33">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45814</v>
       </c>
       <c r="AT4" s="33" t="s">
@@ -2166,7 +2140,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="5" spans="1:77" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" ht="52.5" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>140</v>
       </c>
@@ -2198,7 +2172,7 @@
         <v>83</v>
       </c>
       <c r="K5" s="33">
-        <f ca="1">TODAY()-31</f>
+        <f>TODAY()-31</f>
         <v>45692</v>
       </c>
       <c r="L5" s="34" t="s">
@@ -2238,7 +2212,7 @@
         <v>83</v>
       </c>
       <c r="X5" s="33">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45692</v>
       </c>
       <c r="Y5" s="34" t="s">
@@ -2284,7 +2258,7 @@
         <v>98</v>
       </c>
       <c r="AM5" s="33">
-        <f t="shared" ca="1" si="6"/>
+        <f t="shared" si="6"/>
         <v>46088</v>
       </c>
       <c r="AN5" s="34">
@@ -2300,11 +2274,11 @@
         <v>101</v>
       </c>
       <c r="AR5" s="33">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45692</v>
       </c>
       <c r="AS5" s="33">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45692</v>
       </c>
       <c r="AT5" s="33" t="s">
@@ -2402,7 +2376,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:77" ht="54" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" ht="54" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>146</v>
       </c>
@@ -2434,7 +2408,7 @@
         <v>83</v>
       </c>
       <c r="K6" s="33">
-        <f ca="1">TODAY()+91</f>
+        <f>TODAY()+91</f>
         <v>45814</v>
       </c>
       <c r="L6" s="34" t="s">
@@ -2474,7 +2448,7 @@
         <v>83</v>
       </c>
       <c r="X6" s="33">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45814</v>
       </c>
       <c r="Y6" s="34" t="s">
@@ -2535,11 +2509,11 @@
         <v>101</v>
       </c>
       <c r="AR6" s="33">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45814</v>
       </c>
       <c r="AS6" s="33">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45814</v>
       </c>
       <c r="AT6" s="33" t="s">
@@ -2637,7 +2611,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:77" ht="52.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" ht="52.5" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>151</v>
       </c>
@@ -2669,7 +2643,7 @@
         <v>83</v>
       </c>
       <c r="K7" s="33">
-        <f ca="1">TODAY()-31</f>
+        <f>TODAY()-31</f>
         <v>45692</v>
       </c>
       <c r="L7" s="34" t="s">
@@ -2709,7 +2683,7 @@
         <v>83</v>
       </c>
       <c r="X7" s="33">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45692</v>
       </c>
       <c r="Y7" s="34" t="s">
@@ -2755,7 +2729,7 @@
         <v>98</v>
       </c>
       <c r="AM7" s="33">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AN7" s="34">
@@ -2771,15 +2745,15 @@
         <v>101</v>
       </c>
       <c r="AR7" s="33">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45692</v>
       </c>
       <c r="AS7" s="33">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45692</v>
       </c>
       <c r="AT7" s="33">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AU7" s="34" t="s">
@@ -2874,7 +2848,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:77" ht="54" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="8" ht="54" customHeight="1" spans="1:77" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>158</v>
       </c>
@@ -2906,7 +2880,7 @@
         <v>83</v>
       </c>
       <c r="K8" s="33">
-        <f ca="1">TODAY()-31</f>
+        <f>TODAY()-31</f>
         <v>45692</v>
       </c>
       <c r="L8" s="34" t="s">
@@ -2946,7 +2920,7 @@
         <v>83</v>
       </c>
       <c r="X8" s="33">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" si="1"/>
         <v>45692</v>
       </c>
       <c r="Y8" s="34" t="s">
@@ -2992,7 +2966,7 @@
         <v>98</v>
       </c>
       <c r="AM8" s="33">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AN8" s="34">
@@ -3008,15 +2982,15 @@
         <v>101</v>
       </c>
       <c r="AR8" s="33">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" si="3"/>
         <v>45692</v>
       </c>
       <c r="AS8" s="33">
-        <f t="shared" ca="1" si="4"/>
+        <f t="shared" si="4"/>
         <v>45692</v>
       </c>
       <c r="AT8" s="33">
-        <f ca="1">TODAY()+365</f>
+        <f>TODAY()+365</f>
         <v>46088</v>
       </c>
       <c r="AU8" s="34" t="s">
@@ -3112,8 +3086,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BY8" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:BY8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>